<commit_message>
Complete project handover workflow and configurable summaries
</commit_message>
<xml_diff>
--- a/docs/reference/stackexchange-published-statistics.xlsx
+++ b/docs/reference/stackexchange-published-statistics.xlsx
@@ -15,11 +15,21 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Software Eng. tags" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Read me'!$A$1:$B$9</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Summary'!$A$1:$C$5</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="1">'Summary'!$A$1:$C$5</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'All sites'!$A$1:$P$184</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="2">'All sites'!$1:$1</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="2">'All sites'!$A$1:$P$184</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Stack Overflow tags'!$A$1:$F$101</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="3">'Stack Overflow tags'!$1:$1</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="3">'Stack Overflow tags'!$A$1:$F$101</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Super User tags'!$A$1:$F$51</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="4">'Super User tags'!$1:$1</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="4">'Super User tags'!$A$1:$F$51</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Software Eng. tags'!$A$1:$F$51</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="5">'Software Eng. tags'!$1:$1</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="5">'Software Eng. tags'!$A$1:$F$51</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -539,7 +549,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:B9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
@@ -658,7 +668,17 @@
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B2" r:id="rId1"/>
   </hyperlinks>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <printOptions horizontalCentered="1"/>
+  <pageMargins left="0.25" right="0.25" top="0.5" bottom="0.5" header="0.2" footer="0.2"/>
+  <pageSetup orientation="landscape" paperSize="8" fitToHeight="0" fitToWidth="1"/>
+  <headerFooter>
+    <oddHeader>&amp;C&amp;BRead me</oddHeader>
+    <oddFooter>&amp;CPage &amp;P of &amp;N</oddFooter>
+    <evenHeader/>
+    <evenFooter/>
+    <firstHeader/>
+    <firstFooter/>
+  </headerFooter>
 </worksheet>
 </file>
 
@@ -666,7 +686,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:C5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
@@ -767,7 +787,17 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C4" r:id="rId3"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C5" r:id="rId4"/>
   </hyperlinks>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <printOptions horizontalCentered="1"/>
+  <pageMargins left="0.25" right="0.25" top="0.5" bottom="0.5" header="0.2" footer="0.2"/>
+  <pageSetup orientation="landscape" paperSize="8" fitToHeight="0" fitToWidth="1"/>
+  <headerFooter>
+    <oddHeader>&amp;C&amp;BSummary</oddHeader>
+    <oddFooter>&amp;CPage &amp;P of &amp;N</oddFooter>
+    <evenHeader/>
+    <evenFooter/>
+    <firstHeader/>
+    <firstFooter/>
+  </headerFooter>
   <tableParts count="1">
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId5"/>
   </tableParts>
@@ -778,7 +808,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:P184"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
@@ -13880,7 +13910,17 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C183" r:id="rId182"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C184" r:id="rId183"/>
   </hyperlinks>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <printOptions horizontalCentered="1"/>
+  <pageMargins left="0.25" right="0.25" top="0.5" bottom="0.5" header="0.2" footer="0.2"/>
+  <pageSetup orientation="landscape" paperSize="8" fitToHeight="0" fitToWidth="1"/>
+  <headerFooter>
+    <oddHeader>&amp;C&amp;BAll sites</oddHeader>
+    <oddFooter>&amp;CPage &amp;P of &amp;N</oddFooter>
+    <evenHeader/>
+    <evenFooter/>
+    <firstHeader/>
+    <firstFooter/>
+  </headerFooter>
   <tableParts count="1">
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId184"/>
   </tableParts>
@@ -13891,7 +13931,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:F101"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
@@ -16940,7 +16980,17 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D101" r:id="rId199"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E101" r:id="rId200"/>
   </hyperlinks>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <printOptions horizontalCentered="1"/>
+  <pageMargins left="0.25" right="0.25" top="0.5" bottom="0.5" header="0.2" footer="0.2"/>
+  <pageSetup orientation="landscape" paperSize="8" fitToHeight="0" fitToWidth="1"/>
+  <headerFooter>
+    <oddHeader>&amp;C&amp;BStack Overflow tags</oddHeader>
+    <oddFooter>&amp;CPage &amp;P of &amp;N</oddFooter>
+    <evenHeader/>
+    <evenFooter/>
+    <firstHeader/>
+    <firstFooter/>
+  </headerFooter>
   <tableParts count="1">
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId201"/>
   </tableParts>
@@ -16951,7 +17001,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:F51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
@@ -18500,7 +18550,17 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D51" r:id="rId99"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E51" r:id="rId100"/>
   </hyperlinks>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <printOptions horizontalCentered="1"/>
+  <pageMargins left="0.25" right="0.25" top="0.5" bottom="0.5" header="0.2" footer="0.2"/>
+  <pageSetup orientation="landscape" paperSize="8" fitToHeight="0" fitToWidth="1"/>
+  <headerFooter>
+    <oddHeader>&amp;C&amp;BSuper User tags</oddHeader>
+    <oddFooter>&amp;CPage &amp;P of &amp;N</oddFooter>
+    <evenHeader/>
+    <evenFooter/>
+    <firstHeader/>
+    <firstFooter/>
+  </headerFooter>
   <tableParts count="1">
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId101"/>
   </tableParts>
@@ -18511,7 +18571,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:F51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
@@ -20060,7 +20120,17 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D51" r:id="rId99"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E51" r:id="rId100"/>
   </hyperlinks>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <printOptions horizontalCentered="1"/>
+  <pageMargins left="0.25" right="0.25" top="0.5" bottom="0.5" header="0.2" footer="0.2"/>
+  <pageSetup orientation="landscape" paperSize="8" fitToHeight="0" fitToWidth="1"/>
+  <headerFooter>
+    <oddHeader>&amp;C&amp;BSoftware Eng. tags</oddHeader>
+    <oddFooter>&amp;CPage &amp;P of &amp;N</oddFooter>
+    <evenHeader/>
+    <evenFooter/>
+    <firstHeader/>
+    <firstFooter/>
+  </headerFooter>
   <tableParts count="1">
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId101"/>
   </tableParts>

</xml_diff>